<commit_message>
sheets-r56: the pair of fixtures that pins where a line's ink begins
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GaMTqGsGtQPgZrzgEPeCAB
</commit_message>
<xml_diff>
--- a/dotnet/tests/corpus/features/sheet-band-clip-xlsx.xlsx
+++ b/dotnet/tests/corpus/features/sheet-band-clip-xlsx.xlsx
@@ -4,6 +4,8 @@
   <sheets>
     <sheet name="Areas" sheetId="1" r:id="rId1"/>
     <sheet name="Face" sheetId="2" r:id="rId2"/>
+    <sheet name="Sliver" sheetId="3" r:id="rId3"/>
+    <sheet name="Slice" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -77,4 +79,42 @@
     <oddFooter>&amp;L&amp;"Courier New"FACECODE&amp;CPLAINFACE&amp;R&amp;24BIGFACE</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>BODYCELL</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.32778" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;CTHINBAND</oddHeader>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>BODYCELL</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.35556" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;CWIDEBAND</oddHeader>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>